<commit_message>
fix: normalize iosxe interface commands and aggregate multi-interface evidence
</commit_message>
<xml_diff>
--- a/docs/webhook_v5_family_capability_command_matrix.xlsx
+++ b/docs/webhook_v5_family_capability_command_matrix.xlsx
@@ -101,7 +101,7 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2026-05-11 17:12:45</t>
+          <t xml:space="preserve">2026-05-12 11:31:41</t>
         </is>
       </c>
     </row>
@@ -5034,12 +5034,12 @@
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
@@ -15845,12 +15845,12 @@
       </c>
       <c r="E116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G116" t="inlineStr" s="0">
@@ -17000,12 +17000,12 @@
       </c>
       <c r="E137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G137" t="inlineStr" s="0">
@@ -18155,12 +18155,12 @@
       </c>
       <c r="E158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G158" t="inlineStr" s="0">
@@ -19695,12 +19695,12 @@
       </c>
       <c r="E186" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F186" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G186" t="inlineStr" s="0">
@@ -20850,12 +20850,12 @@
       </c>
       <c r="E207" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F207" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G207" t="inlineStr" s="0">
@@ -22005,12 +22005,12 @@
       </c>
       <c r="E228" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces {interface}</t>
+          <t xml:space="preserve">show interface {interface}</t>
         </is>
       </c>
       <c r="F228" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interfaces Ethernet1/1</t>
+          <t xml:space="preserve">show interface Ethernet1/1</t>
         </is>
       </c>
       <c r="G228" t="inlineStr" s="0">

</xml_diff>

<commit_message>
fix: expand multi-interface circuit utilization evidence
</commit_message>
<xml_diff>
--- a/docs/webhook_v5_family_capability_command_matrix.xlsx
+++ b/docs/webhook_v5_family_capability_command_matrix.xlsx
@@ -101,7 +101,7 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2026-05-12 11:31:41</t>
+          <t xml:space="preserve">2026-05-13 09:52:13</t>
         </is>
       </c>
     </row>
@@ -5034,12 +5034,12 @@
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="0">
@@ -15845,12 +15845,12 @@
       </c>
       <c r="E116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G116" t="inlineStr" s="0">
@@ -17000,12 +17000,12 @@
       </c>
       <c r="E137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G137" t="inlineStr" s="0">
@@ -18155,12 +18155,12 @@
       </c>
       <c r="E158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G158" t="inlineStr" s="0">
@@ -19695,12 +19695,12 @@
       </c>
       <c r="E186" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F186" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G186" t="inlineStr" s="0">
@@ -20850,12 +20850,12 @@
       </c>
       <c r="E207" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F207" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G207" t="inlineStr" s="0">
@@ -22005,12 +22005,12 @@
       </c>
       <c r="E228" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface {interface}</t>
+          <t xml:space="preserve">show interfaces {interface}</t>
         </is>
       </c>
       <c r="F228" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">show interface Ethernet1/1</t>
+          <t xml:space="preserve">show interfaces Ethernet1/1</t>
         </is>
       </c>
       <c r="G228" t="inlineStr" s="0">

</xml_diff>